<commit_message>
feat: adicionando um button de deleta o produto indesejado, em adicionar produto de maneria inteligente
</commit_message>
<xml_diff>
--- a/Estudos_de_python/nfe_27260415342821000183550010000849921077717579.xlsx
+++ b/Estudos_de_python/nfe_27260415342821000183550010000849921077717579.xlsx
@@ -484,16 +484,16 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>43.78</v>
+        <v>49.49</v>
       </c>
       <c r="D2" t="n">
-        <v>72.33</v>
+        <v>83.75</v>
       </c>
       <c r="E2" t="n">
         <v>38.07</v>
       </c>
       <c r="F2" t="n">
-        <v>57.11</v>
+        <v>68.53</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -521,16 +521,16 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>31.27</v>
+        <v>35.35</v>
       </c>
       <c r="D3" t="n">
-        <v>51.66</v>
+        <v>59.82</v>
       </c>
       <c r="E3" t="n">
         <v>27.19</v>
       </c>
       <c r="F3" t="n">
-        <v>40.79</v>
+        <v>48.94</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -558,16 +558,16 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>30.03</v>
+        <v>33.94</v>
       </c>
       <c r="D4" t="n">
-        <v>49.61</v>
+        <v>57.44</v>
       </c>
       <c r="E4" t="n">
         <v>26.11</v>
       </c>
       <c r="F4" t="n">
-        <v>39.16</v>
+        <v>47</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -595,16 +595,16 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>28.14</v>
+        <v>31.81</v>
       </c>
       <c r="D5" t="n">
-        <v>46.49</v>
+        <v>53.83</v>
       </c>
       <c r="E5" t="n">
         <v>24.47</v>
       </c>
       <c r="F5" t="n">
-        <v>36.7</v>
+        <v>44.05</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -632,16 +632,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>30.03</v>
+        <v>33.94</v>
       </c>
       <c r="D6" t="n">
-        <v>49.61</v>
+        <v>57.44</v>
       </c>
       <c r="E6" t="n">
         <v>26.11</v>
       </c>
       <c r="F6" t="n">
-        <v>39.16</v>
+        <v>47</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -669,16 +669,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>39.02</v>
+        <v>44.11</v>
       </c>
       <c r="D7" t="n">
-        <v>64.47</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="E7" t="n">
         <v>33.93</v>
       </c>
       <c r="F7" t="n">
-        <v>50.89</v>
+        <v>61.07</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: ajustando o scraping
</commit_message>
<xml_diff>
--- a/Estudos_de_python/nfe_27260415342821000183550010000849921077717579.xlsx
+++ b/Estudos_de_python/nfe_27260415342821000183550010000849921077717579.xlsx
@@ -423,7 +423,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="239" customWidth="1" min="8" max="8"/>
+    <col width="203" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -502,7 +502,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://carrefourbr.vtexassets.com/arquivos/ids/160997685/da2f6ecf94234ab4bfa574bdda1cad54.jpg?v=638543149740770000</t>
+          <t>https://img.lojasrenner.com.br/item/927427034/zoom/1.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://m.media-amazon.com/images/I/61RTx3xDWSL._AC_SL1500_.jpg</t>
+          <t>https://i.ytimg.com/vi/ySEKAOPnpdE/maxresdefault.jpg</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>http://res.cloudinary.com/beleza-na-web/image/upload/w_297,c_lpad,w_600,h_315/g_south_west,l_label-free-shipping,x_10,y_-60,o_0/v1/imagens/product/E89980/5a70a549-707f-45ec-a006-0f0797be2042-e89980-palette-quarteto-sombras-turbo-8g-1.jpg</t>
+          <t>https://res.cloudinary.com/beleza-na-web/image/upload/w_1500,f_auto,fl_progressive,q_auto:eco,w_800/v1/imagens/product/E55799/d2a3536d-f11d-4841-999a-fbd64b9d7ad4-e55799-paleta-soul-turbo-principal.jpg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">

</xml_diff>